<commit_message>
JP Site Execution & Video URL Verification
</commit_message>
<xml_diff>
--- a/Tests/AboutMarc/AboutMarc_Fail.xlsx
+++ b/Tests/AboutMarc/AboutMarc_Fail.xlsx
@@ -124,86 +124,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>1</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1905000" cy="1905000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId1"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>2</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1905000" cy="1905000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="2" name="Image 2" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId2"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-  <oneCellAnchor>
-    <from>
-      <col>2</col>
-      <colOff>0</colOff>
-      <row>3</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1905000" cy="1905000"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="3" name="Image 3" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId3"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -493,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:D1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="50" customWidth="1" min="1" max="1"/>
@@ -524,59 +444,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="150" customHeight="1">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>https://dev.marcjacobs.com/us-en/about-marc.html</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>https://marcjacobs.bynder.com/match/MJ_Filename/20240920_HISTORY_SLICE_11_MOBILE/?preset=4COL_0</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>No results for url found: consider case sensitivity</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="150" customHeight="1">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>https://dev.marcjacobs.com/us-en/about-marc.html</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>https://cdn.media.amplience.net/i/Marc_Jacobs/SP26_SEARCH_DESKTOP?fmt=auto&amp;w=1600&amp;qlt=50</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>Amplience found in URL</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="150" customHeight="1">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>https://dev.marcjacobs.com/us-en/about-marc.html</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>https://cdn.media.amplience.net/i/Marc_Jacobs/SP26_SEARCH_MOBILE?fmt=auto&amp;w=800&amp;qlt=50</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>Amplience found in URL</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>